<commit_message>
Update job loss phrases in Better alternatives.xlsx per CEFR progression
Agent-Logs-Url: https://github.com/academiaohara/cambridge-exams/sessions/7e8671aa-74f3-49a9-b737-fe9b8a037a6c

Co-authored-by: academiaohara <253255719+academiaohara@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/Social media/Better alternatives.xlsx
+++ b/data/Social media/Better alternatives.xlsx
@@ -495,27 +495,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>She lost her job last month.</t>
+          <t>She lost her job.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>She got fired last month.</t>
+          <t>She became unemployed.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>She was made redundant last month.</t>
+          <t>She was made redundant.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>She faced dismissal last month.</t>
+          <t>She was dismissed.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>She was issued a notice of termination last month.</t>
+          <t>She had her employment terminated.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Better alternatives CSV/XLSX with new expressions and bold formatting
Agent-Logs-Url: https://github.com/academiaohara/cambridge-exams/sessions/8f767985-3393-40ac-9abc-9e04a6e40657

Co-authored-by: academiaohara <253255719+academiaohara@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/Social media/Better alternatives.xlsx
+++ b/data/Social media/Better alternatives.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="25" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -495,27 +495,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>She lost her job.</t>
+          <t>She **lost her job**.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>She became unemployed.</t>
+          <t>She was **made redundant**.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>She was made redundant.</t>
+          <t>She was **dismissed**.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>She was dismissed.</t>
+          <t>She was **let go** following a strategic realignment.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>She had her employment terminated.</t>
+          <t>She was **outplaced** as part of a workforce reduction.</t>
         </is>
       </c>
     </row>
@@ -527,1561 +527,1625 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>I'm happy.</t>
+          <t>She was **very happy**.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>I'm really happy about it.</t>
+          <t>She was **really pleased**.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>I'm thrilled with the news.</t>
+          <t>She was **over the moon**.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>I couldn't be more pleased.</t>
+          <t>She was **absolutely ecstatic**.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>I'm absolutely overjoyed; it's beyond my expectations</t>
+          <t>She was in a state of **unadulterated bliss**.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>To express disappointment</t>
+          <t>To express tiredness</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>I'm sad.</t>
+          <t>He was **very tired**.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>I'm a bit disappointed.</t>
+          <t>He was **exhausted**.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>It's disappointing, honestly.</t>
+          <t>He was **worn out**.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>I'm rather dissatisfied with how things turned out.</t>
+          <t>He **could barely keep his eyes open**.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>It's a profound letdown, given the effort invested.</t>
+          <t>He was **running on fumes**.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>To make a suggestion</t>
+          <t>To express anger</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Let's go.</t>
+          <t>He was **angry**.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Why don't we go?</t>
+          <t>He **got really angry**.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>We could consider going.</t>
+          <t>He was **livid**.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>I'd suggest we explore other options.</t>
+          <t>He **couldn't contain his anger**.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>It might be prudent to consider an alternative course of action.</t>
+          <t>He was **seething with rage**.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>To apologize</t>
+          <t>To express disappointment</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Sorry.</t>
+          <t>I'm sad.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>I'm so sorry.</t>
+          <t>I'm a bit disappointed.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>I apologize for that.</t>
+          <t>It's disappointing, honestly.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>I'd like to offer my sincere apologies.</t>
+          <t>I'm rather dissatisfied with how things turned out.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>I deeply regret any inconvenience this may have caused.</t>
+          <t>It's a profound letdown, given the effort invested.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>To ask for permission</t>
+          <t>To make a suggestion</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Can I go?</t>
+          <t>Let's go.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Is it okay if I go?</t>
+          <t>Why don't we go?</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Would it be possible for me to go?</t>
+          <t>We could consider going.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>I'd like to request permission to go.</t>
+          <t>I'd suggest we explore other options.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>I seek your authorization to proceed.</t>
+          <t>It might be prudent to consider an alternative course of action.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>To give an opinion</t>
+          <t>To apologize</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>I think it's good.</t>
+          <t>Sorry.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>In my opinion, it's good.</t>
+          <t>I'm so sorry.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>I'd say it's a solid option.</t>
+          <t>I apologize for that.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>From my perspective, it's quite effective.</t>
+          <t>I'd like to offer my sincere apologies.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>It would appear to be the most judicious approach.</t>
+          <t>I deeply regret any inconvenience this may have caused.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>To describe a problem</t>
+          <t>To ask for permission</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>It doesn't work.</t>
+          <t>Can I go?</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>There's a problem with it.</t>
+          <t>Is it okay if I go?</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>We're experiencing some issues.</t>
+          <t>Would it be possible for me to go?</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>We've encountered a technical setback.</t>
+          <t>I'd like to request permission to go.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>We're facing a significant operational impediment.</t>
+          <t>I seek your authorization to proceed.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>To talk about the weather</t>
+          <t>To give an opinion</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>It's sunny.</t>
+          <t>I think it's good.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>It's a beautiful day.</t>
+          <t>In my opinion, it's good.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>What lovely weather we're having.</t>
+          <t>I'd say it's a solid option.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>The weather is exceptionally pleasant.</t>
+          <t>From my perspective, it's quite effective.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>We're being treated to a spell of glorious sunshine.</t>
+          <t>It would appear to be the most judicious approach.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>To make a request</t>
+          <t>To describe a problem</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Help me.</t>
+          <t>It doesn't work.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Could you help me?</t>
+          <t>There's a problem with it.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>I was wondering if you could help.</t>
+          <t>We're experiencing some issues.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Would you be able to assist me?</t>
+          <t>We've encountered a technical setback.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>I would greatly appreciate your assistance with this.</t>
+          <t>We're facing a significant operational impediment.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>To express uncertainty</t>
+          <t>To talk about the weather</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>I don't know.</t>
+          <t>It's sunny.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>I'm not sure.</t>
+          <t>It's a beautiful day.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>I'm not entirely certain.</t>
+          <t>What lovely weather we're having.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>I'm still unclear on that point.</t>
+          <t>The weather is exceptionally pleasant.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>There remains a degree of ambiguity surrounding the matter.</t>
+          <t>We're being treated to a spell of glorious sunshine.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>To give bad news</t>
+          <t>To make a request</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>It's bad.</t>
+          <t>Help me.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>I have some bad news.</t>
+          <t>Could you help me?</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Unfortunately, I've got some bad news.</t>
+          <t>I was wondering if you could help.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>I regret to inform you that things haven't gone as planned.</t>
+          <t>Would you be able to assist me?</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>It is with some reluctance that I convey this unfavorable development.</t>
+          <t>I would greatly appreciate your assistance with this.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>To show interest</t>
+          <t>To express uncertainty</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Oh, cool.</t>
+          <t>I don't know.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>That sounds interesting.</t>
+          <t>I'm not sure.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>How fascinating.</t>
+          <t>I'm not entirely certain.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>That's quite intriguing.</t>
+          <t>I'm still unclear on that point.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>I find that exceptionally compelling.</t>
+          <t>There remains a degree of ambiguity surrounding the matter.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>To end a conversation</t>
+          <t>To give bad news</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Bye.</t>
+          <t>It's bad.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Nice talking to you.</t>
+          <t>I have some bad news.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>It was great chatting.</t>
+          <t>Unfortunately, I've got some bad news.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>I've really enjoyed our conversation.</t>
+          <t>I regret to inform you that things haven't gone as planned.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>It's been a genuine pleasure speaking with you; let's reconnect soon</t>
+          <t>It is with some reluctance that I convey this unfavorable development.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>To describe ability</t>
+          <t>To show interest</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>I can swim.</t>
+          <t>Oh, cool.</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>I'm able to swim.</t>
+          <t>That sounds interesting.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>I possess the ability to swim.</t>
+          <t>How fascinating.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>I'm quite proficient at swimming.</t>
+          <t>That's quite intriguing.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>I have attained a high level of competency in swimming.</t>
+          <t>I find that exceptionally compelling.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>To complain</t>
+          <t>To end a conversation</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>This is bad.</t>
+          <t>Bye.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>I'm not happy with this.</t>
+          <t>Nice talking to you.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>This isn't quite what I expected.</t>
+          <t>It was great chatting.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>I'm afraid this falls short of the agreed standard.</t>
+          <t>I've really enjoyed our conversation.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>This does not align with the specifications previously established.</t>
+          <t>It's been a genuine pleasure speaking with you; let's reconnect soon</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>To give instructions</t>
+          <t>To describe ability</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Do this.</t>
+          <t>I can swim.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>First, you do this.</t>
+          <t>I'm able to swim.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>The first step is to do this.</t>
+          <t>I possess the ability to swim.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>To begin, you'll need to carry out this step.</t>
+          <t>I'm quite proficient at swimming.</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Commence by executing this procedure with precision.</t>
+          <t>I have attained a high level of competency in swimming.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>To make a promise</t>
+          <t>To complain</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>I'll do it.</t>
+          <t>This is bad.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>I promise I'll do it.</t>
+          <t>I'm not happy with this.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>You have my word I'll do it.</t>
+          <t>This isn't quite what I expected.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>I assure you I'll take care of it.</t>
+          <t>I'm afraid this falls short of the agreed standard.</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>I give you my solemn commitment that it will be addressed.</t>
+          <t>This does not align with the specifications previously established.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>To agree</t>
+          <t>To give instructions</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Yes.</t>
+          <t>Do this.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>I agree.</t>
+          <t>First, you do this.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>That makes sense.</t>
+          <t>The first step is to do this.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>I'm in full agreement.</t>
+          <t>To begin, you'll need to carry out this step.</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>I wholeheartedly concur with that perspective.</t>
+          <t>Commence by executing this procedure with precision.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>To disagree</t>
+          <t>To make a promise</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>No.</t>
+          <t>I'll do it.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>I don't think so.</t>
+          <t>I promise I'll do it.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>I'm not sure I agree.</t>
+          <t>You have my word I'll do it.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>I see it differently, I'm afraid.</t>
+          <t>I assure you I'll take care of it.</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>I respectfully beg to differ on that point.</t>
+          <t>I give you my solemn commitment that it will be addressed.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>To share something online</t>
+          <t>To agree</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>I shared a photo.</t>
+          <t>Yes.</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>I posted a photo online.</t>
+          <t>I agree.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>I shared some content on my profile.</t>
+          <t>That makes sense.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>I uploaded and distributed the content across my social channels.</t>
+          <t>I'm in full agreement.</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>I disseminated the material via my digital platforms for broader reach.</t>
+          <t>I wholeheartedly concur with that perspective.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>To say something is popular online</t>
+          <t>To disagree</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>It's very popular.</t>
+          <t>No.</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>It's going viral.</t>
+          <t>I don't think so.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>It's gained a lot of traction online.</t>
+          <t>I'm not sure I agree.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>It's garnered significant engagement across platforms.</t>
+          <t>I see it differently, I'm afraid.</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>It has achieved widespread virality and cross-platform resonance.</t>
+          <t>I respectfully beg to differ on that point.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>To follow someone online</t>
+          <t>To share something online</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>I like her page.</t>
+          <t>I shared a photo.</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>I follow her account.</t>
+          <t>I posted a photo online.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>I subscribe to her content regularly.</t>
+          <t>I shared some content on my profile.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>I keep up with her posts and engage with her online presence.</t>
+          <t>I uploaded and distributed the content across my social channels.</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>I actively monitor her digital output and engage with her online persona.</t>
+          <t>I disseminated the material via my digital platforms for broader reach.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>To comment on a post</t>
+          <t>To say something is popular online</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>I wrote a comment.</t>
+          <t>It's very popular.</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>I left a comment on that post.</t>
+          <t>It's going viral.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>I weighed in on the discussion with a comment.</t>
+          <t>It's gained a lot of traction online.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>I added my thoughts to the thread below the post.</t>
+          <t>It's garnered significant engagement across platforms.</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>I contributed my perspective to the online discourse beneath that publication.</t>
+          <t>It has achieved widespread virality and cross-platform resonance.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>To describe a trending topic</t>
+          <t>To follow someone online</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Everyone is talking about it.</t>
+          <t>I like her page.</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>It's everywhere right now.</t>
+          <t>I follow her account.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>It's currently a hot topic online.</t>
+          <t>I subscribe to her content regularly.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>It's dominating the conversation across social media platforms.</t>
+          <t>I keep up with her posts and engage with her online presence.</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>It has permeated the collective discourse and captured widespread public attention.</t>
+          <t>I actively monitor her digital output and engage with her online persona.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>To describe a photo or image</t>
+          <t>To comment on a post</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Nice photo.</t>
+          <t>I wrote a comment.</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>That's a great picture.</t>
+          <t>I left a comment on that post.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>That's a really striking image.</t>
+          <t>I weighed in on the discussion with a comment.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>What a beautifully composed photograph.</t>
+          <t>I added my thoughts to the thread below the post.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>The composition and lighting of this image are truly exceptional.</t>
+          <t>I contributed my perspective to the online discourse beneath that publication.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>To agree with content online</t>
+          <t>To describe a trending topic</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>I like this.</t>
+          <t>Everyone is talking about it.</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>This is so true.</t>
+          <t>It's everywhere right now.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>I can totally relate to this.</t>
+          <t>It's currently a hot topic online.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>This resonates deeply with my own experience.</t>
+          <t>It's dominating the conversation across social media platforms.</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>The sentiments expressed here align precisely with my own convictions.</t>
+          <t>It has permeated the collective discourse and captured widespread public attention.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>To describe someone's online presence</t>
+          <t>To describe a photo or image</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>She posts a lot.</t>
+          <t>Nice photo.</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>She's very active on social media.</t>
+          <t>That's a great picture.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>She has a strong online presence.</t>
+          <t>That's a really striking image.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>She maintains a highly visible and engaged digital profile.</t>
+          <t>What a beautifully composed photograph.</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>She has cultivated an extensive and influential digital footprint across multiple platforms.</t>
+          <t>The composition and lighting of this image are truly exceptional.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>To describe something as fake or untrue</t>
+          <t>To agree with content online</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>It's not real.</t>
+          <t>I like this.</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>I don't think that's true.</t>
+          <t>This is so true.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>That seems to be misinformation.</t>
+          <t>I can totally relate to this.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>I have serious doubts about the veracity of that claim.</t>
+          <t>This resonates deeply with my own experience.</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>The authenticity of that assertion appears to be fundamentally compromised.</t>
+          <t>The sentiments expressed here align precisely with my own convictions.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>To talk about unfollowing someone online</t>
+          <t>To describe someone's online presence</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>I deleted him.</t>
+          <t>She posts a lot.</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>I unfollowed him online.</t>
+          <t>She's very active on social media.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>I decided to unfollow and distance myself online.</t>
+          <t>She has a strong online presence.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>I felt it necessary to remove him from my social media contacts.</t>
+          <t>She maintains a highly visible and engaged digital profile.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>I resolved to sever all digital connections with him across social platforms.</t>
+          <t>She has cultivated an extensive and influential digital footprint across multiple platforms.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>To react to offensive online content</t>
+          <t>To describe something as fake or untrue</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>That's not nice.</t>
+          <t>It's not real.</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>That's really offensive.</t>
+          <t>I don't think that's true.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>I find that kind of content quite inappropriate.</t>
+          <t>That seems to be misinformation.</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Such material is wholly unacceptable and potentially harmful.</t>
+          <t>I have serious doubts about the veracity of that claim.</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Content of this nature is not only objectionable but potentially injurious to public discourse.</t>
+          <t>The authenticity of that assertion appears to be fundamentally compromised.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>To talk about screen time</t>
+          <t>To talk about unfollowing someone online</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>I use my phone a lot.</t>
+          <t>I deleted him.</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>I spend a lot of time on my phone.</t>
+          <t>I unfollowed him online.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>I tend to be glued to my phone most of the day.</t>
+          <t>I decided to unfollow and distance myself online.</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>My screen time has reached a level I find rather excessive.</t>
+          <t>I felt it necessary to remove him from my social media contacts.</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>My level of digital device engagement has escalated to a degree I find somewhat disconcerting.</t>
+          <t>I resolved to sever all digital connections with him across social platforms.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>To express gratitude</t>
+          <t>To react to offensive online content</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Thank you!</t>
+          <t>That's not nice.</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Thanks a lot, I really appreciate it.</t>
+          <t>That's really offensive.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>I'm really grateful for your help.</t>
+          <t>I find that kind of content quite inappropriate.</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>I'd like to express my sincere gratitude for your support.</t>
+          <t>Such material is wholly unacceptable and potentially harmful.</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>I am profoundly indebted to you for your invaluable assistance.</t>
+          <t>Content of this nature is not only objectionable but potentially injurious to public discourse.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>To express surprise</t>
+          <t>To talk about screen time</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Wow!</t>
+          <t>I use my phone a lot.</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>I can't believe it!</t>
+          <t>I spend a lot of time on my phone.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>That's really unexpected.</t>
+          <t>I tend to be glued to my phone most of the day.</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>I must say, that's quite astonishing.</t>
+          <t>My screen time has reached a level I find rather excessive.</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>I find myself utterly taken aback by this turn of events.</t>
+          <t>My level of digital device engagement has escalated to a degree I find somewhat disconcerting.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>To talk about future plans</t>
+          <t>To express gratitude</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>I will go to Paris.</t>
+          <t>Thank you!</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>I'm planning to go to Paris.</t>
+          <t>Thanks a lot, I really appreciate it.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>I'm looking forward to visiting Paris in the near future.</t>
+          <t>I'm really grateful for your help.</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>I have every intention of travelling to Paris in the coming months.</t>
+          <t>I'd like to express my sincere gratitude for your support.</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>I am fully committed to undertaking a visit to Paris at the earliest opportunity.</t>
+          <t>I am profoundly indebted to you for your invaluable assistance.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>To express obligation</t>
+          <t>To express surprise</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>I must do it.</t>
+          <t>Wow!</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>I have to do it.</t>
+          <t>I can't believe it!</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>I'm obliged to get it done.</t>
+          <t>That's really unexpected.</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>I'm under an obligation to see this through.</t>
+          <t>I must say, that's quite astonishing.</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>I find myself compelled by circumstances to fulfil this commitment.</t>
+          <t>I find myself utterly taken aback by this turn of events.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>To ask for advice</t>
+          <t>To talk about future plans</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>What do I do?</t>
+          <t>I will go to Paris.</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>What do you think I should do?</t>
+          <t>I'm planning to go to Paris.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Could you give me some advice on this?</t>
+          <t>I'm looking forward to visiting Paris in the near future.</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>I'd welcome your guidance on how to handle this situation.</t>
+          <t>I have every intention of travelling to Paris in the coming months.</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>I would be most grateful for your considered counsel on this matter.</t>
+          <t>I am fully committed to undertaking a visit to Paris at the earliest opportunity.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>To express worry or concern</t>
+          <t>To express obligation</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>I'm scared.</t>
+          <t>I must do it.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>I'm a bit worried about it.</t>
+          <t>I have to do it.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>I'm quite concerned about how things might turn out.</t>
+          <t>I'm obliged to get it done.</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>I have some reservations about the possible outcome.</t>
+          <t>I'm under an obligation to see this through.</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>I find myself gripped by considerable apprehension regarding the potential repercussions.</t>
+          <t>I find myself compelled by circumstances to fulfil this commitment.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>To encourage someone</t>
+          <t>To ask for advice</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>You can do it!</t>
+          <t>What do I do?</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Keep going, you're doing great!</t>
+          <t>What do you think I should do?</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Don't give up, you're making real progress.</t>
+          <t>Could you give me some advice on this?</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>I have every confidence that you'll pull through.</t>
+          <t>I'd welcome your guidance on how to handle this situation.</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Your perseverance is commendable; I have no doubt you will prevail.</t>
+          <t>I would be most grateful for your considered counsel on this matter.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>To recommend something</t>
+          <t>To express worry or concern</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>This is good.</t>
+          <t>I'm scared.</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>You should try this.</t>
+          <t>I'm a bit worried about it.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>I'd really recommend giving this a go.</t>
+          <t>I'm quite concerned about how things might turn out.</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>I strongly suggest you consider this option.</t>
+          <t>I have some reservations about the possible outcome.</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>I would wholeheartedly advocate for this particular course of action.</t>
+          <t>I find myself gripped by considerable apprehension regarding the potential repercussions.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>To invite someone</t>
+          <t>To encourage someone</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Come with me.</t>
+          <t>You can do it!</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Do you want to come with me?</t>
+          <t>Keep going, you're doing great!</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>I'd love it if you could join me.</t>
+          <t>Don't give up, you're making real progress.</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>I would be delighted if you could accompany me.</t>
+          <t>I have every confidence that you'll pull through.</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>It would be a great honour if you would consider gracing us with your presence.</t>
+          <t>Your perseverance is commendable; I have no doubt you will prevail.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>To describe a personal achievement</t>
+          <t>To recommend something</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>I did it!</t>
+          <t>This is good.</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>I managed to do it!</t>
+          <t>You should try this.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>I successfully pulled it off.</t>
+          <t>I'd really recommend giving this a go.</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>I'm pleased to report that I've accomplished what I set out to do.</t>
+          <t>I strongly suggest you consider this option.</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>I have successfully brought this endeavour to a most satisfactory conclusion.</t>
+          <t>I would wholeheartedly advocate for this particular course of action.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>To describe something difficult</t>
+          <t>To invite someone</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>It's hard.</t>
+          <t>Come with me.</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>It's quite difficult.</t>
+          <t>Do you want to come with me?</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>It's more challenging than I expected.</t>
+          <t>I'd love it if you could join me.</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>This poses a considerable challenge.</t>
+          <t>I would be delighted if you could accompany me.</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>This undertaking proves to be a formidable and complex endeavour.</t>
+          <t>It would be a great honour if you would consider gracing us with your presence.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>To talk about preferences</t>
+          <t>To describe a personal achievement</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>I like cats.</t>
+          <t>I did it!</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>I prefer cats to dogs.</t>
+          <t>I managed to do it!</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>I have a preference for cats over dogs.</t>
+          <t>I successfully pulled it off.</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>I tend to favour cats, finding them more suitable to my lifestyle.</t>
+          <t>I'm pleased to report that I've accomplished what I set out to do.</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>I hold a marked predisposition towards feline companionship over canine alternatives.</t>
+          <t>I have successfully brought this endeavour to a most satisfactory conclusion.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>To express contrast</t>
+          <t>To describe something difficult</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>But it's also good.</t>
+          <t>It's hard.</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>On the other hand, it has some benefits.</t>
+          <t>It's quite difficult.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>That said, there are some positive aspects worth noting.</t>
+          <t>It's more challenging than I expected.</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Nevertheless, it would be remiss not to acknowledge certain merits.</t>
+          <t>This poses a considerable challenge.</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Notwithstanding the above, one must concede the existence of countervailing virtues.</t>
+          <t>This undertaking proves to be a formidable and complex endeavour.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>To give an example</t>
+          <t>To talk about preferences</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Like this.</t>
+          <t>I like cats.</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>For example, this one.</t>
+          <t>I prefer cats to dogs.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>To illustrate, consider this case.</t>
+          <t>I have a preference for cats over dogs.</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>To cite a pertinent example, one might consider...</t>
+          <t>I tend to favour cats, finding them more suitable to my lifestyle.</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>By way of exemplification, one may draw attention to the following instance.</t>
+          <t>I hold a marked predisposition towards feline companionship over canine alternatives.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>To summarize or conclude</t>
+          <t>To express contrast</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>So, it's good.</t>
+          <t>But it's also good.</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>In short, it works well.</t>
+          <t>On the other hand, it has some benefits.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>To sum up, it's been a positive experience.</t>
+          <t>That said, there are some positive aspects worth noting.</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>In conclusion, the overall outcome has been favourable.</t>
+          <t>Nevertheless, it would be remiss not to acknowledge certain merits.</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>To distil the matter to its essence, the results have proven most propitious.</t>
+          <t>Notwithstanding the above, one must concede the existence of countervailing virtues.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>To say you miss someone</t>
+          <t>To give an example</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>I miss you.</t>
+          <t>Like this.</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>I've been thinking about you a lot.</t>
+          <t>For example, this one.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>I really miss having you around.</t>
+          <t>To illustrate, consider this case.</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Your absence has left quite a void.</t>
+          <t>To cite a pertinent example, one might consider...</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>One cannot overstate the extent to which your presence is sorely missed.</t>
+          <t>By way of exemplification, one may draw attention to the following instance.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>To tell someone to stop doing something</t>
+          <t>To summarize or conclude</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Stop it!</t>
+          <t>So, it's good.</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Please don't do that.</t>
+          <t>In short, it works well.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>I'd appreciate it if you stopped doing that.</t>
+          <t>To sum up, it's been a positive experience.</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>I must ask you to refrain from that behaviour.</t>
+          <t>In conclusion, the overall outcome has been favourable.</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>I would respectfully urge you to desist from this course of conduct forthwith.</t>
+          <t>To distil the matter to its essence, the results have proven most propitious.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>To say you miss someone</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>I miss you.</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>I've been thinking about you a lot.</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>I really miss having you around.</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Your absence has left quite a void.</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>One cannot overstate the extent to which your presence is sorely missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>To tell someone to stop doing something</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Stop it!</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Please don't do that.</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>I'd appreciate it if you stopped doing that.</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>I must ask you to refrain from that behaviour.</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>I would respectfully urge you to desist from this course of conduct forthwith.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t>To describe feeling overwhelmed</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>I have too much to do.</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>I'm feeling a bit overwhelmed.</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t>I've got a lot on my plate at the moment.</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t>I'm finding it increasingly difficult to manage all my commitments.</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="F53" t="inlineStr">
         <is>
           <t>I find myself beset by an accumulation of obligations that threatens to exceed my capacity to cope.</t>
         </is>

</xml_diff>

<commit_message>
Remove wrongly-added rows and bold key vocabulary in all existing rows
Agent-Logs-Url: https://github.com/academiaohara/cambridge-exams/sessions/dbd17859-71d8-4993-8d63-b3ba4a278667

Co-authored-by: academiaohara <253255719+academiaohara@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/Social media/Better alternatives.xlsx
+++ b/data/Social media/Better alternatives.xlsx
@@ -554,1603 +554,1541 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>To express tiredness</t>
+          <t>To express disappointment</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>He was **very tired**.</t>
+          <t>I'm **sad**.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>He was **exhausted**.</t>
+          <t>I'm **a bit disappointed**.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>He was **worn out**.</t>
+          <t>I'm absolutely **gutted**.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>He **could barely keep his eyes open**.</t>
+          <t>I'm **rather disheartened** by the outcome.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>He was **running on fumes**.</t>
+          <t>I find the outcome **profoundly disheartening**.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>To express anger</t>
+          <t>To make a suggestion</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>He was **angry**.</t>
+          <t>**Let's go**.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>He **got really angry**.</t>
+          <t>**Why don't we** go?</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>He was **livid**.</t>
+          <t>We **could consider** going.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>He **couldn't contain his anger**.</t>
+          <t>I'd **suggest** we explore other options.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>He was **seething with rage**.</t>
+          <t>It might be **prudent to consider** an alternative course of action.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>To express disappointment</t>
+          <t>To apologize</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>I'm sad.</t>
+          <t>**Sorry**.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>I'm a bit disappointed.</t>
+          <t>I'm **so sorry**.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>It's disappointing, honestly.</t>
+          <t>I **apologize** for that.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>I'm rather dissatisfied with how things turned out.</t>
+          <t>I'd like to offer my **sincere apologies**.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>It's a profound letdown, given the effort invested.</t>
+          <t>I **deeply regret** any inconvenience this may have caused.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>To make a suggestion</t>
+          <t>To ask for permission</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Let's go.</t>
+          <t>**Can I** go?</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Why don't we go?</t>
+          <t>**Is it okay if** I go?</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>We could consider going.</t>
+          <t>**Would it be possible for** me to go?</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>I'd suggest we explore other options.</t>
+          <t>I'd like to **request permission** to go.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>It might be prudent to consider an alternative course of action.</t>
+          <t>I **seek your authorization** to proceed.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>To apologize</t>
+          <t>To give an opinion</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Sorry.</t>
+          <t>I **think** it's good.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>I'm so sorry.</t>
+          <t>**In my opinion**, it's good.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>I apologize for that.</t>
+          <t>I'd **say** it's a solid option.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>I'd like to offer my sincere apologies.</t>
+          <t>**From my perspective**, it's quite effective.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>I deeply regret any inconvenience this may have caused.</t>
+          <t>It would appear to be the most **judicious** approach.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>To ask for permission</t>
+          <t>To describe a problem</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Can I go?</t>
+          <t>It **doesn't work**.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Is it okay if I go?</t>
+          <t>There's a **problem** with it.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Would it be possible for me to go?</t>
+          <t>We're **experiencing some issues**.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>I'd like to request permission to go.</t>
+          <t>We've **encountered a technical setback**.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>I seek your authorization to proceed.</t>
+          <t>We're facing a significant **operational impediment**.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>To give an opinion</t>
+          <t>To talk about the weather</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>I think it's good.</t>
+          <t>It's **sunny**.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>In my opinion, it's good.</t>
+          <t>It's a **beautiful day**.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>I'd say it's a solid option.</t>
+          <t>What **lovely weather** we're having.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>From my perspective, it's quite effective.</t>
+          <t>The weather is **exceptionally pleasant**.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>It would appear to be the most judicious approach.</t>
+          <t>We're being treated to a **spell of glorious sunshine**.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>To describe a problem</t>
+          <t>To make a request</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>It doesn't work.</t>
+          <t>**Help** me.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>There's a problem with it.</t>
+          <t>**Could you** help me?</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>We're experiencing some issues.</t>
+          <t>I was wondering **if you could** help.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>We've encountered a technical setback.</t>
+          <t>**Would you be able to** assist me?</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>We're facing a significant operational impediment.</t>
+          <t>I would **greatly appreciate** your assistance with this.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>To talk about the weather</t>
+          <t>To express uncertainty</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>It's sunny.</t>
+          <t>I **don't know**.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>It's a beautiful day.</t>
+          <t>I'm **not sure**.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>What lovely weather we're having.</t>
+          <t>I'm **not entirely certain**.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>The weather is exceptionally pleasant.</t>
+          <t>I'm **still unclear** on that point.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>We're being treated to a spell of glorious sunshine.</t>
+          <t>There remains a degree of **ambiguity** surrounding the matter.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>To make a request</t>
+          <t>To give bad news</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Help me.</t>
+          <t>It's **bad**.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Could you help me?</t>
+          <t>I have some **bad news**.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>I was wondering if you could help.</t>
+          <t>**Unfortunately**, I've got some bad news.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Would you be able to assist me?</t>
+          <t>I **regret to inform** you that things haven't gone as planned.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>I would greatly appreciate your assistance with this.</t>
+          <t>It is with some **reluctance** that I convey this unfavorable development.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>To express uncertainty</t>
+          <t>To show interest</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>I don't know.</t>
+          <t>**Oh, cool**.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>I'm not sure.</t>
+          <t>That sounds **interesting**.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>I'm not entirely certain.</t>
+          <t>How **fascinating**.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>I'm still unclear on that point.</t>
+          <t>That's quite **intriguing**.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>There remains a degree of ambiguity surrounding the matter.</t>
+          <t>I find that **exceptionally compelling**.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>To give bad news</t>
+          <t>To end a conversation</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>It's bad.</t>
+          <t>**Bye**.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>I have some bad news.</t>
+          <t>**Nice talking** to you.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Unfortunately, I've got some bad news.</t>
+          <t>It was **great chatting**.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>I regret to inform you that things haven't gone as planned.</t>
+          <t>I've **really enjoyed** our conversation.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>It is with some reluctance that I convey this unfavorable development.</t>
+          <t>It's been a **genuine pleasure** speaking with you; let's reconnect soon.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>To show interest</t>
+          <t>To describe ability</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Oh, cool.</t>
+          <t>I **can** swim.</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>That sounds interesting.</t>
+          <t>I'm **able to** swim.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>How fascinating.</t>
+          <t>I **possess the ability** to swim.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>That's quite intriguing.</t>
+          <t>I'm quite **proficient** at swimming.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>I find that exceptionally compelling.</t>
+          <t>I have **attained a high level of competency** in swimming.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>To end a conversation</t>
+          <t>To complain</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Bye.</t>
+          <t>This is **bad**.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Nice talking to you.</t>
+          <t>I'm **not happy** with this.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>It was great chatting.</t>
+          <t>This isn't quite **what I expected**.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>I've really enjoyed our conversation.</t>
+          <t>I'm afraid this **falls short** of the agreed standard.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>It's been a genuine pleasure speaking with you; let's reconnect soon</t>
+          <t>This does not **align with** the specifications previously established.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>To describe ability</t>
+          <t>To give instructions</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>I can swim.</t>
+          <t>**Do this**.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>I'm able to swim.</t>
+          <t>**First**, you do this.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>I possess the ability to swim.</t>
+          <t>The **first step** is to do this.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>I'm quite proficient at swimming.</t>
+          <t>**To begin**, you'll need to carry out this step.</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>I have attained a high level of competency in swimming.</t>
+          <t>**Commence** by executing this procedure with precision.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>To complain</t>
+          <t>To make a promise</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>This is bad.</t>
+          <t>I'll **do it**.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>I'm not happy with this.</t>
+          <t>I **promise** I'll do it.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>This isn't quite what I expected.</t>
+          <t>You have my **word** I'll do it.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>I'm afraid this falls short of the agreed standard.</t>
+          <t>I **assure** you I'll take care of it.</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>This does not align with the specifications previously established.</t>
+          <t>I give you my **solemn commitment** that it will be addressed.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>To give instructions</t>
+          <t>To agree</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Do this.</t>
+          <t>**Yes**.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>First, you do this.</t>
+          <t>I **agree**.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>The first step is to do this.</t>
+          <t>That **makes sense**.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>To begin, you'll need to carry out this step.</t>
+          <t>I'm in **full agreement**.</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Commence by executing this procedure with precision.</t>
+          <t>I **wholeheartedly concur** with that perspective.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>To make a promise</t>
+          <t>To disagree</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>I'll do it.</t>
+          <t>**No**.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>I promise I'll do it.</t>
+          <t>I **don't think so**.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>You have my word I'll do it.</t>
+          <t>I'm **not sure I agree**.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>I assure you I'll take care of it.</t>
+          <t>I **see it differently**, I'm afraid.</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>I give you my solemn commitment that it will be addressed.</t>
+          <t>I **respectfully beg to differ** on that point.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>To agree</t>
+          <t>To share something online</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Yes.</t>
+          <t>I **shared** a photo.</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>I agree.</t>
+          <t>I **posted** a photo online.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>That makes sense.</t>
+          <t>I **shared some content** on my profile.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>I'm in full agreement.</t>
+          <t>I **uploaded and distributed** the content across my social channels.</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>I wholeheartedly concur with that perspective.</t>
+          <t>I **disseminated** the material via my digital platforms for broader reach.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>To disagree</t>
+          <t>To say something is popular online</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>No.</t>
+          <t>It's **very popular**.</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>I don't think so.</t>
+          <t>It's **going viral**.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>I'm not sure I agree.</t>
+          <t>It's **gained a lot of traction** online.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>I see it differently, I'm afraid.</t>
+          <t>It's **garnered significant engagement** across platforms.</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>I respectfully beg to differ on that point.</t>
+          <t>It has achieved **widespread virality** and cross-platform resonance.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>To share something online</t>
+          <t>To follow someone online</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>I shared a photo.</t>
+          <t>I **like** her page.</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>I posted a photo online.</t>
+          <t>I **follow** her account.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>I shared some content on my profile.</t>
+          <t>I **subscribe to** her content regularly.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>I uploaded and distributed the content across my social channels.</t>
+          <t>I **keep up with** her posts and engage with her online presence.</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>I disseminated the material via my digital platforms for broader reach.</t>
+          <t>I actively **monitor her digital output** and engage with her online persona.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>To say something is popular online</t>
+          <t>To comment on a post</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>It's very popular.</t>
+          <t>I **wrote a comment**.</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>It's going viral.</t>
+          <t>I **left a comment** on that post.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>It's gained a lot of traction online.</t>
+          <t>I **weighed in on** the discussion with a comment.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>It's garnered significant engagement across platforms.</t>
+          <t>I **added my thoughts** to the thread below the post.</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>It has achieved widespread virality and cross-platform resonance.</t>
+          <t>I **contributed my perspective** to the online discourse beneath that publication.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>To follow someone online</t>
+          <t>To describe a trending topic</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>I like her page.</t>
+          <t>**Everyone is talking** about it.</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>I follow her account.</t>
+          <t>It's **everywhere** right now.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>I subscribe to her content regularly.</t>
+          <t>It's currently a **hot topic** online.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>I keep up with her posts and engage with her online presence.</t>
+          <t>It's **dominating the conversation** across social media platforms.</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>I actively monitor her digital output and engage with her online persona.</t>
+          <t>It has **permeated the collective discourse** and captured widespread public attention.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>To comment on a post</t>
+          <t>To describe a photo or image</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>I wrote a comment.</t>
+          <t>**Nice photo**.</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>I left a comment on that post.</t>
+          <t>That's a **great picture**.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>I weighed in on the discussion with a comment.</t>
+          <t>That's a really **striking image**.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>I added my thoughts to the thread below the post.</t>
+          <t>What a **beautifully composed** photograph.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>I contributed my perspective to the online discourse beneath that publication.</t>
+          <t>The **composition and lighting** of this image are truly exceptional.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>To describe a trending topic</t>
+          <t>To agree with content online</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Everyone is talking about it.</t>
+          <t>I **like** this.</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>It's everywhere right now.</t>
+          <t>This is **so true**.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>It's currently a hot topic online.</t>
+          <t>I can **totally relate** to this.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>It's dominating the conversation across social media platforms.</t>
+          <t>This **resonates deeply** with my own experience.</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>It has permeated the collective discourse and captured widespread public attention.</t>
+          <t>The sentiments expressed here **align precisely** with my own convictions.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>To describe a photo or image</t>
+          <t>To describe someone's online presence</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Nice photo.</t>
+          <t>She **posts a lot**.</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>That's a great picture.</t>
+          <t>She's **very active** on social media.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>That's a really striking image.</t>
+          <t>She has a **strong online presence**.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>What a beautifully composed photograph.</t>
+          <t>She **maintains a highly visible** and engaged digital profile.</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>The composition and lighting of this image are truly exceptional.</t>
+          <t>She has **cultivated an extensive and influential digital footprint** across multiple platforms.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>To agree with content online</t>
+          <t>To describe something as fake or untrue</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>I like this.</t>
+          <t>It's **not real**.</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>This is so true.</t>
+          <t>I don't think **that's true**.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>I can totally relate to this.</t>
+          <t>That seems to be **misinformation**.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>This resonates deeply with my own experience.</t>
+          <t>I have serious doubts about the **veracity** of that claim.</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>The sentiments expressed here align precisely with my own convictions.</t>
+          <t>The **authenticity** of that assertion appears to be fundamentally compromised.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>To describe someone's online presence</t>
+          <t>To talk about unfollowing someone online</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>She posts a lot.</t>
+          <t>I **deleted** him.</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>She's very active on social media.</t>
+          <t>I **unfollowed** him online.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>She has a strong online presence.</t>
+          <t>I decided to **unfollow and distance** myself online.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>She maintains a highly visible and engaged digital profile.</t>
+          <t>I felt it necessary to **remove him** from my social media contacts.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>She has cultivated an extensive and influential digital footprint across multiple platforms.</t>
+          <t>I resolved to **sever all digital connections** with him across social platforms.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>To describe something as fake or untrue</t>
+          <t>To react to offensive online content</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>It's not real.</t>
+          <t>That's **not nice**.</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>I don't think that's true.</t>
+          <t>That's **really offensive**.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>That seems to be misinformation.</t>
+          <t>I find that kind of content **quite inappropriate**.</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>I have serious doubts about the veracity of that claim.</t>
+          <t>Such material is **wholly unacceptable** and potentially harmful.</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>The authenticity of that assertion appears to be fundamentally compromised.</t>
+          <t>Content of this nature is not only **objectionable** but potentially injurious to public discourse.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>To talk about unfollowing someone online</t>
+          <t>To talk about screen time</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>I deleted him.</t>
+          <t>I use my phone **a lot**.</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>I unfollowed him online.</t>
+          <t>I **spend a lot of time** on my phone.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>I decided to unfollow and distance myself online.</t>
+          <t>I tend to be **glued to** my phone most of the day.</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>I felt it necessary to remove him from my social media contacts.</t>
+          <t>My screen time has reached a level I find **rather excessive**.</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>I resolved to sever all digital connections with him across social platforms.</t>
+          <t>My level of **digital device engagement** has escalated to a degree I find somewhat disconcerting.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>To react to offensive online content</t>
+          <t>To express gratitude</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>That's not nice.</t>
+          <t>**Thank you**!</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>That's really offensive.</t>
+          <t>**Thanks a lot**, I really appreciate it.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>I find that kind of content quite inappropriate.</t>
+          <t>I'm really **grateful** for your help.</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Such material is wholly unacceptable and potentially harmful.</t>
+          <t>I'd like to express my **sincere gratitude** for your support.</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Content of this nature is not only objectionable but potentially injurious to public discourse.</t>
+          <t>I am **profoundly indebted** to you for your invaluable assistance.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>To talk about screen time</t>
+          <t>To express surprise</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>I use my phone a lot.</t>
+          <t>**Wow**!</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>I spend a lot of time on my phone.</t>
+          <t>I **can't believe** it!</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>I tend to be glued to my phone most of the day.</t>
+          <t>That's really **unexpected**.</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>My screen time has reached a level I find rather excessive.</t>
+          <t>I must say, that's quite **astonishing**.</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>My level of digital device engagement has escalated to a degree I find somewhat disconcerting.</t>
+          <t>I find myself utterly **taken aback** by this turn of events.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>To express gratitude</t>
+          <t>To talk about future plans</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Thank you!</t>
+          <t>I **will go** to Paris.</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Thanks a lot, I really appreciate it.</t>
+          <t>I'm **planning to go** to Paris.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>I'm really grateful for your help.</t>
+          <t>I'm **looking forward to** visiting Paris in the near future.</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>I'd like to express my sincere gratitude for your support.</t>
+          <t>I have **every intention of** travelling to Paris in the coming months.</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>I am profoundly indebted to you for your invaluable assistance.</t>
+          <t>I am **fully committed to** undertaking a visit to Paris at the earliest opportunity.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>To express surprise</t>
+          <t>To express obligation</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Wow!</t>
+          <t>I **must** do it.</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>I can't believe it!</t>
+          <t>I **have to** do it.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>That's really unexpected.</t>
+          <t>I'm **obliged** to get it done.</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>I must say, that's quite astonishing.</t>
+          <t>I'm **under an obligation** to see this through.</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>I find myself utterly taken aback by this turn of events.</t>
+          <t>I find myself **compelled by circumstances** to fulfil this commitment.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>To talk about future plans</t>
+          <t>To ask for advice</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>I will go to Paris.</t>
+          <t>What do I **do**?</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>I'm planning to go to Paris.</t>
+          <t>What do you think I **should do**?</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>I'm looking forward to visiting Paris in the near future.</t>
+          <t>Could you give me some **advice** on this?</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>I have every intention of travelling to Paris in the coming months.</t>
+          <t>I'd **welcome your guidance** on how to handle this situation.</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>I am fully committed to undertaking a visit to Paris at the earliest opportunity.</t>
+          <t>I would be most grateful for your **considered counsel** on this matter.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>To express obligation</t>
+          <t>To express worry or concern</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>I must do it.</t>
+          <t>I'm **scared**.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>I have to do it.</t>
+          <t>I'm **a bit worried** about it.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>I'm obliged to get it done.</t>
+          <t>I'm quite **concerned** about how things might turn out.</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>I'm under an obligation to see this through.</t>
+          <t>I have some **reservations** about the possible outcome.</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>I find myself compelled by circumstances to fulfil this commitment.</t>
+          <t>I find myself gripped by considerable **apprehension** regarding the potential repercussions.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>To ask for advice</t>
+          <t>To encourage someone</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>What do I do?</t>
+          <t>**You can do it**!</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>What do you think I should do?</t>
+          <t>**Keep going**, you're doing great!</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Could you give me some advice on this?</t>
+          <t>**Don't give up**, you're making real progress.</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>I'd welcome your guidance on how to handle this situation.</t>
+          <t>I have **every confidence** that you'll pull through.</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>I would be most grateful for your considered counsel on this matter.</t>
+          <t>Your **perseverance** is commendable; I have no doubt you will prevail.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>To express worry or concern</t>
+          <t>To recommend something</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>I'm scared.</t>
+          <t>This is **good**.</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>I'm a bit worried about it.</t>
+          <t>You **should try** this.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>I'm quite concerned about how things might turn out.</t>
+          <t>I'd really **recommend** giving this a go.</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>I have some reservations about the possible outcome.</t>
+          <t>I **strongly suggest** you consider this option.</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>I find myself gripped by considerable apprehension regarding the potential repercussions.</t>
+          <t>I would **wholeheartedly advocate** for this particular course of action.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>To encourage someone</t>
+          <t>To invite someone</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>You can do it!</t>
+          <t>**Come with me**.</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Keep going, you're doing great!</t>
+          <t>Do you **want to come** with me?</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Don't give up, you're making real progress.</t>
+          <t>I'd **love it** if you could join me.</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>I have every confidence that you'll pull through.</t>
+          <t>I would be **delighted** if you could accompany me.</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Your perseverance is commendable; I have no doubt you will prevail.</t>
+          <t>It would be a **great honour** if you would consider gracing us with your presence.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>To recommend something</t>
+          <t>To describe a personal achievement</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>This is good.</t>
+          <t>**I did it**!</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>You should try this.</t>
+          <t>I **managed to do it**!</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>I'd really recommend giving this a go.</t>
+          <t>I **successfully pulled it off**.</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>I strongly suggest you consider this option.</t>
+          <t>I'm pleased to report that I've **accomplished** what I set out to do.</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>I would wholeheartedly advocate for this particular course of action.</t>
+          <t>I have **successfully brought this endeavour** to a most satisfactory conclusion.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>To invite someone</t>
+          <t>To describe something difficult</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Come with me.</t>
+          <t>It's **hard**.</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Do you want to come with me?</t>
+          <t>It's quite **difficult**.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>I'd love it if you could join me.</t>
+          <t>It's **more challenging** than I expected.</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>I would be delighted if you could accompany me.</t>
+          <t>This **poses a considerable challenge**.</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>It would be a great honour if you would consider gracing us with your presence.</t>
+          <t>This undertaking proves to be a **formidable and complex** endeavour.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>To describe a personal achievement</t>
+          <t>To talk about preferences</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>I did it!</t>
+          <t>I **like** cats.</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>I managed to do it!</t>
+          <t>I **prefer** cats to dogs.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>I successfully pulled it off.</t>
+          <t>I have a **preference for** cats over dogs.</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>I'm pleased to report that I've accomplished what I set out to do.</t>
+          <t>I tend to **favour** cats, finding them more suitable to my lifestyle.</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>I have successfully brought this endeavour to a most satisfactory conclusion.</t>
+          <t>I hold a **marked predisposition** towards feline companionship over canine alternatives.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>To describe something difficult</t>
+          <t>To express contrast</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>It's hard.</t>
+          <t>But it's **also** good.</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>It's quite difficult.</t>
+          <t>**On the other hand**, it has some benefits.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>It's more challenging than I expected.</t>
+          <t>**That said**, there are some positive aspects worth noting.</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>This poses a considerable challenge.</t>
+          <t>**Nevertheless**, it would be remiss not to acknowledge certain merits.</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>This undertaking proves to be a formidable and complex endeavour.</t>
+          <t>**Notwithstanding the above**, one must concede the existence of countervailing virtues.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>To talk about preferences</t>
+          <t>To give an example</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>I like cats.</t>
+          <t>**Like this**.</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>I prefer cats to dogs.</t>
+          <t>**For example**, this one.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>I have a preference for cats over dogs.</t>
+          <t>**To illustrate**, consider this case.</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>I tend to favour cats, finding them more suitable to my lifestyle.</t>
+          <t>**To cite a pertinent example**, one might consider...</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>I hold a marked predisposition towards feline companionship over canine alternatives.</t>
+          <t>**By way of exemplification**, one may draw attention to the following instance.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>To express contrast</t>
+          <t>To summarize or conclude</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>But it's also good.</t>
+          <t>So, it's **good**.</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>On the other hand, it has some benefits.</t>
+          <t>**In short**, it works well.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>That said, there are some positive aspects worth noting.</t>
+          <t>**To sum up**, it's been a positive experience.</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Nevertheless, it would be remiss not to acknowledge certain merits.</t>
+          <t>**In conclusion**, the overall outcome has been favourable.</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Notwithstanding the above, one must concede the existence of countervailing virtues.</t>
+          <t>**To distil the matter to its essence**, the results have proven most propitious.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>To give an example</t>
+          <t>To say you miss someone</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Like this.</t>
+          <t>I **miss you**.</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>For example, this one.</t>
+          <t>I've been **thinking about** you a lot.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>To illustrate, consider this case.</t>
+          <t>I really **miss having you around**.</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>To cite a pertinent example, one might consider...</t>
+          <t>Your **absence has left quite a void**.</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>By way of exemplification, one may draw attention to the following instance.</t>
+          <t>One cannot overstate the extent to which your presence is **sorely missed**.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>To summarize or conclude</t>
+          <t>To tell someone to stop doing something</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>So, it's good.</t>
+          <t>**Stop it**!</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>In short, it works well.</t>
+          <t>Please **don't do that**.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>To sum up, it's been a positive experience.</t>
+          <t>I'd **appreciate it** if you stopped doing that.</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>In conclusion, the overall outcome has been favourable.</t>
+          <t>I must ask you to **refrain from** that behaviour.</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>To distil the matter to its essence, the results have proven most propitious.</t>
+          <t>I would respectfully urge you to **desist from** this course of conduct forthwith.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>To say you miss someone</t>
+          <t>To describe feeling overwhelmed</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>I miss you.</t>
+          <t>I have **too much to do**.</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>I've been thinking about you a lot.</t>
+          <t>I'm feeling **a bit overwhelmed**.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>I really miss having you around.</t>
+          <t>I've got **a lot on my plate** at the moment.</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Your absence has left quite a void.</t>
+          <t>I'm finding it **increasingly difficult** to manage all my commitments.</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>One cannot overstate the extent to which your presence is sorely missed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>To tell someone to stop doing something</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Stop it!</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Please don't do that.</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>I'd appreciate it if you stopped doing that.</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>I must ask you to refrain from that behaviour.</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>I would respectfully urge you to desist from this course of conduct forthwith.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>To describe feeling overwhelmed</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>I have too much to do.</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>I'm feeling a bit overwhelmed.</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>I've got a lot on my plate at the moment.</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>I'm finding it increasingly difficult to manage all my commitments.</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>I find myself beset by an accumulation of obligations that threatens to exceed my capacity to cope.</t>
-        </is>
-      </c>
-    </row>
+          <t>I find myself **beset by** an accumulation of obligations that threatens to exceed my capacity to cope.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52"/>
+    <row r="53"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>